<commit_message>
refine: remove Layer 1 references, move report to bottom, add Q&A pairs
Remove Layer 1 from page header, glossary title and presentation slide 1.
Move Physical Report output below tabs at full width with larger text.
Break chat transcript expander into labeled steps with Step 2 marked as
examples. Add 5 new describe Q&A pairs: no speculation on play style,
no prior knowledge, SkillCorner data source, P90 explanation, no named
player comparisons. Update presentation: white text on player slides,
examples note on Step 2 slide.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/describe/Physical.xlsx
+++ b/data/describe/Physical.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1028,6 +1028,66 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Should you speculate about a player's playing style, tactical role, or team system based on their physical data?</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>No. Physical data tells you what a player can and cannot do physically — it does not tell you how the team plays, what role the coach has assigned them, or why their output looks the way it does. Do not speculate about playing style, tactical systems, or team context. Stick strictly to describing the physical profile: what is strong, what is weak, and what kind of physical athlete the player is. Let the coaching staff draw their own conclusions about how the physical data fits into their tactical picture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Should you use your own knowledge about a player when writing their physical profile?</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>No. You must only use the data provided in the physical profile description. Do not reference anything you know about the player from outside this data — their reputation, transfer history, injury record, playing style, or career trajectory. The profile should read identically whether the player is a global star or an unknown. If the data says a player has poor speed, report poor speed, regardless of what you might believe about them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>What is SkillCorner and where does the physical data come from?</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SkillCorner provides physical tracking data derived from broadcast footage using computer vision, not from GPS vests or wearable devices. This means the data is collected non-invasively from match broadcasts and covers players across many leagues without requiring club cooperation. The metrics — speeds, accelerations, distances, changes of direction — are all estimated from optical tracking of player movement during competitive matches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>What does P90 mean and why is it used?</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>P90 means the value is normalised to per 90 minutes of playing time. This controls for the fact that players play different numbers of minutes across a season. A player who has played 2,000 minutes will naturally accumulate more total distance than one who has played 900 minutes, but their per-90 figures can be compared fairly. Always treat P90 metrics as rates, not totals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Should you compare a player to other named players in their physical profile?</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>No. Never reference other players by name when describing a physical profile. Do not say things like 'similar to Mbappé' or 'unlike most centre-backs such as Van Dijk'. Each profile should describe the player purely in terms of their own data relative to their position group. Comparisons to named individuals introduce bias and are outside the scope of the data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>